<commit_message>
Update template with post modeling changes (#138)
* modify desk review template

* update condo desk_review
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damajor\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3991A33C-F26A-4683-BCC0-EBDF0F0957AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4682E70-921D-4671-8E7E-5BEA648BF6A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -553,12 +553,6 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Total AV</t>
-  </si>
-  <si>
-    <t>AV Difference</t>
-  </si>
-  <si>
     <t>Sale Num. Parcels 1</t>
   </si>
   <si>
@@ -583,28 +577,35 @@
     <t>Recent Assessable Permit</t>
   </si>
   <si>
-    <t>Min MV</t>
-  </si>
-  <si>
-    <t>Average MV</t>
-  </si>
-  <si>
-    <t>Max MV</t>
-  </si>
-  <si>
-    <t>Average MV Difference</t>
+    <t>Total MV</t>
+  </si>
+  <si>
+    <t>MV Difference</t>
+  </si>
+  <si>
+    <t>Average of MV Difference</t>
+  </si>
+  <si>
+    <t>Min of Total MV</t>
+  </si>
+  <si>
+    <t>Average of Total MV</t>
+  </si>
+  <si>
+    <t>Max of Total MV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="[$$-409]#,##0"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -855,7 +856,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -985,6 +986,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -992,7 +994,68 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="20">
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="[$$-409]#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="[$$-409]#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1012,7 +1075,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46063.730929745368" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{71C4991D-10B4-4CFF-8A35-19A87D2DBFEA}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46072.631774189816" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{71C4991D-10B4-4CFF-8A35-19A87D2DBFEA}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_range"/>
   </cacheSource>
@@ -1175,10 +1238,10 @@
     <cacheField name="Recent Assessable Permit" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Total AV" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="AV Difference" numFmtId="0">
+    <cacheField name="Total MV" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="MV Difference" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
   </cacheFields>
@@ -1347,12 +1410,38 @@
     </i>
   </colItems>
   <dataFields count="5">
-    <dataField name="Min MV" fld="52" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average MV" fld="52" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max MV" fld="52" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average MV Difference" fld="53" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Min of Total MV" fld="52" subtotal="min" baseField="2" baseItem="0" numFmtId="169"/>
+    <dataField name="Average of Total MV" fld="52" subtotal="average" baseField="2" baseItem="0" numFmtId="169"/>
+    <dataField name="Max of Total MV" fld="52" subtotal="max" baseField="2" baseItem="0" numFmtId="169"/>
+    <dataField name="Average of MV Difference" fld="53" subtotal="average" baseField="2" baseItem="0" numFmtId="169"/>
     <dataField name="Average YoY ∆ %" fld="23" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
+  <formats count="2">
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="4" selected="0">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="4">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1662,52 +1751,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BK1048575"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BK6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15.375" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="11.5" customWidth="1"/>
-    <col min="4" max="4" width="42.58203125" customWidth="1"/>
-    <col min="5" max="5" width="16.58203125" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" style="11" customWidth="1"/>
-    <col min="9" max="10" width="11.83203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.625" customWidth="1"/>
+    <col min="5" max="5" width="16.625" customWidth="1"/>
+    <col min="6" max="6" width="14.375" customWidth="1"/>
+    <col min="7" max="7" width="15.375" customWidth="1"/>
+    <col min="8" max="8" width="13.875" style="11" customWidth="1"/>
+    <col min="9" max="10" width="11.875" style="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" style="10" customWidth="1"/>
-    <col min="12" max="13" width="10.83203125" style="10" customWidth="1"/>
-    <col min="14" max="14" width="9.08203125" style="11" customWidth="1"/>
-    <col min="15" max="15" width="13.58203125" style="15" customWidth="1"/>
-    <col min="16" max="17" width="11.58203125" style="10" customWidth="1"/>
-    <col min="18" max="18" width="13.58203125" style="10" customWidth="1"/>
+    <col min="12" max="13" width="10.875" style="10" customWidth="1"/>
+    <col min="14" max="14" width="9.125" style="11" customWidth="1"/>
+    <col min="15" max="15" width="13.625" style="15" customWidth="1"/>
+    <col min="16" max="17" width="11.625" style="10" customWidth="1"/>
+    <col min="18" max="18" width="13.625" style="10" customWidth="1"/>
     <col min="19" max="19" width="11" style="10"/>
-    <col min="20" max="21" width="10.83203125" style="10" customWidth="1"/>
-    <col min="22" max="22" width="11.58203125" style="11" customWidth="1"/>
+    <col min="20" max="21" width="10.875" style="10" customWidth="1"/>
+    <col min="22" max="22" width="11.625" style="11" customWidth="1"/>
     <col min="23" max="23" width="11" style="12"/>
     <col min="24" max="25" width="11" style="11"/>
-    <col min="26" max="26" width="21.08203125" style="11" customWidth="1"/>
+    <col min="26" max="26" width="21.125" style="11" customWidth="1"/>
     <col min="27" max="27" width="13" customWidth="1"/>
     <col min="28" max="28" width="13" style="10" customWidth="1"/>
-    <col min="29" max="29" width="18.58203125" style="10" customWidth="1"/>
+    <col min="29" max="29" width="18.625" style="10" customWidth="1"/>
     <col min="30" max="32" width="13" style="16" customWidth="1"/>
     <col min="33" max="33" width="13" style="10" customWidth="1"/>
-    <col min="34" max="35" width="18.58203125" style="10" customWidth="1"/>
+    <col min="34" max="35" width="18.625" style="10" customWidth="1"/>
     <col min="36" max="36" width="13" style="16" customWidth="1"/>
     <col min="39" max="40" width="11" style="13"/>
-    <col min="41" max="41" width="16.58203125" style="13" customWidth="1"/>
-    <col min="42" max="42" width="12.83203125" customWidth="1"/>
-    <col min="43" max="45" width="15.58203125" customWidth="1"/>
-    <col min="46" max="46" width="12.58203125" customWidth="1"/>
-    <col min="47" max="47" width="13.08203125" customWidth="1"/>
-    <col min="48" max="48" width="14.08203125" customWidth="1"/>
+    <col min="41" max="41" width="16.625" style="13" customWidth="1"/>
+    <col min="42" max="42" width="12.875" customWidth="1"/>
+    <col min="43" max="45" width="15.625" customWidth="1"/>
+    <col min="46" max="46" width="12.625" customWidth="1"/>
+    <col min="47" max="47" width="13.125" customWidth="1"/>
+    <col min="48" max="48" width="14.125" customWidth="1"/>
     <col min="50" max="51" width="14" customWidth="1"/>
     <col min="52" max="52" width="13" customWidth="1"/>
     <col min="53" max="53" width="7.75" hidden="1" customWidth="1"/>
-    <col min="54" max="54" width="9.33203125" hidden="1" customWidth="1"/>
-    <col min="55" max="55" width="15.08203125" customWidth="1"/>
+    <col min="54" max="54" width="9.375" hidden="1" customWidth="1"/>
+    <col min="55" max="55" width="15.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:63" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="5"/>
       <c r="B1" s="38"/>
       <c r="C1" s="38"/>
@@ -1772,7 +1861,7 @@
       <c r="BJ1" s="5"/>
       <c r="BK1" s="5"/>
     </row>
-    <row r="2" spans="1:63" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1812,7 +1901,7 @@
       <c r="AN2"/>
       <c r="AO2"/>
     </row>
-    <row r="3" spans="1:63" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>29</v>
       </c>
@@ -1853,7 +1942,7 @@
       <c r="AN3"/>
       <c r="AO3"/>
     </row>
-    <row r="4" spans="1:63" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="H4"/>
       <c r="I4"/>
@@ -1887,7 +1976,7 @@
       <c r="AN4"/>
       <c r="AO4"/>
     </row>
-    <row r="5" spans="1:63" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.25">
       <c r="B5" s="33" t="s">
         <v>48</v>
       </c>
@@ -1954,7 +2043,7 @@
       <c r="BA5" s="18"/>
       <c r="BB5" s="18"/>
     </row>
-    <row r="6" spans="1:63" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:63" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
@@ -2028,7 +2117,7 @@
         <v>3</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Z6" s="3" t="s">
         <v>53</v>
@@ -2046,7 +2135,7 @@
         <v>16</v>
       </c>
       <c r="AE6" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="AF6" s="3" t="s">
         <v>17</v>
@@ -2061,7 +2150,7 @@
         <v>19</v>
       </c>
       <c r="AJ6" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="AK6" s="3" t="s">
         <v>27</v>
@@ -2076,13 +2165,13 @@
         <v>32</v>
       </c>
       <c r="AO6" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AP6" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="AR6" s="9" t="s">
         <v>31</v>
@@ -2109,185 +2198,14 @@
         <v>23</v>
       </c>
       <c r="AZ6" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BB6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="BA6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="BB6" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="1048519" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048519" s="13"/>
-    </row>
-    <row r="1048520" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048520" s="13"/>
-    </row>
-    <row r="1048521" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048521" s="13"/>
-    </row>
-    <row r="1048522" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048522" s="13"/>
-    </row>
-    <row r="1048523" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048523" s="13"/>
-    </row>
-    <row r="1048524" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048524" s="13"/>
-    </row>
-    <row r="1048525" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048525" s="13"/>
-    </row>
-    <row r="1048526" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048526" s="13"/>
-    </row>
-    <row r="1048527" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048527" s="13"/>
-    </row>
-    <row r="1048528" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048528" s="13"/>
-    </row>
-    <row r="1048529" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048529" s="13"/>
-    </row>
-    <row r="1048530" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048530" s="13"/>
-    </row>
-    <row r="1048531" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048531" s="13"/>
-    </row>
-    <row r="1048532" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048532" s="13"/>
-    </row>
-    <row r="1048533" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048533" s="13"/>
-    </row>
-    <row r="1048534" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048534" s="13"/>
-    </row>
-    <row r="1048535" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048535" s="13"/>
-    </row>
-    <row r="1048536" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048536" s="13"/>
-    </row>
-    <row r="1048537" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048537" s="13"/>
-    </row>
-    <row r="1048538" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048538" s="13"/>
-    </row>
-    <row r="1048539" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048539" s="13"/>
-    </row>
-    <row r="1048540" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048540" s="13"/>
-    </row>
-    <row r="1048541" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048541" s="13"/>
-    </row>
-    <row r="1048542" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048542" s="13"/>
-    </row>
-    <row r="1048543" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048543" s="13"/>
-    </row>
-    <row r="1048544" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048544" s="13"/>
-    </row>
-    <row r="1048545" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048545" s="13"/>
-    </row>
-    <row r="1048546" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048546" s="13"/>
-    </row>
-    <row r="1048547" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048547" s="13"/>
-    </row>
-    <row r="1048548" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048548" s="13"/>
-    </row>
-    <row r="1048549" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048549" s="13"/>
-    </row>
-    <row r="1048550" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048550" s="13"/>
-    </row>
-    <row r="1048551" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048551" s="13"/>
-    </row>
-    <row r="1048552" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048552" s="13"/>
-    </row>
-    <row r="1048553" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048553" s="13"/>
-    </row>
-    <row r="1048554" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048554" s="13"/>
-    </row>
-    <row r="1048555" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048555" s="13"/>
-    </row>
-    <row r="1048556" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048556" s="13"/>
-    </row>
-    <row r="1048557" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048557" s="13"/>
-    </row>
-    <row r="1048558" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048558" s="13"/>
-    </row>
-    <row r="1048559" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048559" s="13"/>
-    </row>
-    <row r="1048560" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048560" s="13"/>
-    </row>
-    <row r="1048561" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048561" s="13"/>
-    </row>
-    <row r="1048562" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048562" s="13"/>
-    </row>
-    <row r="1048563" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048563" s="13"/>
-    </row>
-    <row r="1048564" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048564" s="13"/>
-    </row>
-    <row r="1048565" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048565" s="13"/>
-    </row>
-    <row r="1048566" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048566" s="13"/>
-    </row>
-    <row r="1048567" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048567" s="13"/>
-    </row>
-    <row r="1048568" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048568" s="13"/>
-    </row>
-    <row r="1048569" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048569" s="13"/>
-    </row>
-    <row r="1048570" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048570" s="13"/>
-    </row>
-    <row r="1048571" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048571" s="13"/>
-    </row>
-    <row r="1048572" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048572" s="13"/>
-    </row>
-    <row r="1048573" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048573" s="13"/>
-    </row>
-    <row r="1048574" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048574" s="13"/>
-    </row>
-    <row r="1048575" spans="38:38" x14ac:dyDescent="0.35">
-      <c r="AL1048575" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2309,23 +2227,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M1048573"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="7.58203125" customWidth="1"/>
-    <col min="3" max="3" width="42.58203125" customWidth="1"/>
-    <col min="4" max="4" width="16.58203125" customWidth="1"/>
-    <col min="5" max="6" width="11.58203125" customWidth="1"/>
-    <col min="7" max="7" width="12.58203125" customWidth="1"/>
+    <col min="1" max="1" width="15.375" customWidth="1"/>
+    <col min="2" max="2" width="7.625" customWidth="1"/>
+    <col min="3" max="3" width="42.625" customWidth="1"/>
+    <col min="4" max="4" width="16.625" customWidth="1"/>
+    <col min="5" max="6" width="11.625" customWidth="1"/>
+    <col min="7" max="7" width="12.625" customWidth="1"/>
     <col min="8" max="8" width="26" style="10" customWidth="1"/>
-    <col min="9" max="9" width="31.83203125" style="11" customWidth="1"/>
+    <col min="9" max="9" width="31.875" style="11" customWidth="1"/>
     <col min="10" max="10" width="11" style="12"/>
     <col min="11" max="11" width="11" style="11"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="13" max="13" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="B1" s="38" t="s">
         <v>44</v>
       </c>
@@ -2339,14 +2257,14 @@
       <c r="J1"/>
       <c r="K1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="H2"/>
       <c r="I2"/>
       <c r="J2"/>
       <c r="K2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B3" s="50" t="s">
         <v>48</v>
       </c>
@@ -2366,7 +2284,7 @@
       </c>
       <c r="M3" s="49"/>
     </row>
-    <row r="4" spans="1:13" ht="31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>38</v>
       </c>
@@ -2406,177 +2324,6 @@
       <c r="M4" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="1048517" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048517" s="13"/>
-    </row>
-    <row r="1048518" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048518" s="13"/>
-    </row>
-    <row r="1048519" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048519" s="13"/>
-    </row>
-    <row r="1048520" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048520" s="13"/>
-    </row>
-    <row r="1048521" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048521" s="13"/>
-    </row>
-    <row r="1048522" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048522" s="13"/>
-    </row>
-    <row r="1048523" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048523" s="13"/>
-    </row>
-    <row r="1048524" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048524" s="13"/>
-    </row>
-    <row r="1048525" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048525" s="13"/>
-    </row>
-    <row r="1048526" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048526" s="13"/>
-    </row>
-    <row r="1048527" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048527" s="13"/>
-    </row>
-    <row r="1048528" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048528" s="13"/>
-    </row>
-    <row r="1048529" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048529" s="13"/>
-    </row>
-    <row r="1048530" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048530" s="13"/>
-    </row>
-    <row r="1048531" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048531" s="13"/>
-    </row>
-    <row r="1048532" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048532" s="13"/>
-    </row>
-    <row r="1048533" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048533" s="13"/>
-    </row>
-    <row r="1048534" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048534" s="13"/>
-    </row>
-    <row r="1048535" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048535" s="13"/>
-    </row>
-    <row r="1048536" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048536" s="13"/>
-    </row>
-    <row r="1048537" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048537" s="13"/>
-    </row>
-    <row r="1048538" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048538" s="13"/>
-    </row>
-    <row r="1048539" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048539" s="13"/>
-    </row>
-    <row r="1048540" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048540" s="13"/>
-    </row>
-    <row r="1048541" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048541" s="13"/>
-    </row>
-    <row r="1048542" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048542" s="13"/>
-    </row>
-    <row r="1048543" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048543" s="13"/>
-    </row>
-    <row r="1048544" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048544" s="13"/>
-    </row>
-    <row r="1048545" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048545" s="13"/>
-    </row>
-    <row r="1048546" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048546" s="13"/>
-    </row>
-    <row r="1048547" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048547" s="13"/>
-    </row>
-    <row r="1048548" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048548" s="13"/>
-    </row>
-    <row r="1048549" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048549" s="13"/>
-    </row>
-    <row r="1048550" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048550" s="13"/>
-    </row>
-    <row r="1048551" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048551" s="13"/>
-    </row>
-    <row r="1048552" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048552" s="13"/>
-    </row>
-    <row r="1048553" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048553" s="13"/>
-    </row>
-    <row r="1048554" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048554" s="13"/>
-    </row>
-    <row r="1048555" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048555" s="13"/>
-    </row>
-    <row r="1048556" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048556" s="13"/>
-    </row>
-    <row r="1048557" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048557" s="13"/>
-    </row>
-    <row r="1048558" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048558" s="13"/>
-    </row>
-    <row r="1048559" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048559" s="13"/>
-    </row>
-    <row r="1048560" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048560" s="13"/>
-    </row>
-    <row r="1048561" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048561" s="13"/>
-    </row>
-    <row r="1048562" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048562" s="13"/>
-    </row>
-    <row r="1048563" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048563" s="13"/>
-    </row>
-    <row r="1048564" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048564" s="13"/>
-    </row>
-    <row r="1048565" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048565" s="13"/>
-    </row>
-    <row r="1048566" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048566" s="13"/>
-    </row>
-    <row r="1048567" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048567" s="13"/>
-    </row>
-    <row r="1048568" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048568" s="13"/>
-    </row>
-    <row r="1048569" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048569" s="13"/>
-    </row>
-    <row r="1048570" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048570" s="13"/>
-    </row>
-    <row r="1048571" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048571" s="13"/>
-    </row>
-    <row r="1048572" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048572" s="13"/>
-    </row>
-    <row r="1048573" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M1048573" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2594,18 +2341,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{468F4264-9F60-48E3-A5EA-D04C0BA089E2}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.4140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.9140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.58203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.875" style="51" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.625" style="51" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.125" style="51" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.125" style="51" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="B1" s="38" t="s">
         <v>56</v>
       </c>
@@ -2615,44 +2362,36 @@
       <c r="F1" s="38"/>
       <c r="G1" s="38"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="51" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="C3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3" t="s">
-        <v>73</v>
-      </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
       <c r="F4" s="22"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
       <c r="F5" s="22"/>
     </row>
   </sheetData>

</xml_diff>